<commit_message>
fix(FCC): the empty-Home DOORS (founder finding — no visible way in)
Home's no-data state is now the designed two-door layout: Import a file from your brokerage →
/import-holdings · Add something by hand → Net worth · Connect your first account shown HONESTLY
as 'coming soon' (never hidden) · the retired-paycheck fast path leads when that's the intent ·
the what-you'll-see promise list · guided questions kept as a quiet link · draft resume kept.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/finwise-device-test-build41.xlsx
+++ b/docs/finwise-device-test-build41.xlsx
@@ -1,15 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10703"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/palakjain/Vibe_Coding/finwise/docs/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC3F4004-385A-B844-8F7A-F07B70663A9B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="240" yWindow="20" windowWidth="16100" windowHeight="9660" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Build 41 walk" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -238,8 +257,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -340,13 +359,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -384,7 +411,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -418,6 +445,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -452,9 +480,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -627,28 +656,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E26"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="4.7109375" customWidth="1"/>
-    <col min="2" max="2" width="42.7109375" customWidth="1"/>
-    <col min="3" max="3" width="62.7109375" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" customWidth="1"/>
-    <col min="5" max="5" width="50.7109375" customWidth="1"/>
+    <col min="1" max="1" width="88.33203125" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" customWidth="1"/>
+    <col min="3" max="3" width="62.6640625" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="50.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:5" ht="19" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:5">
+    <row r="2" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5">
+    <row r="4" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3" t="s">
         <v>2</v>
       </c>
@@ -665,7 +694,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:5">
+    <row r="5" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="4" t="s">
         <v>7</v>
       </c>
@@ -678,7 +707,7 @@
       <c r="D5" s="5"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" spans="1:5">
+    <row r="6" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="4" t="s">
         <v>10</v>
       </c>
@@ -691,7 +720,7 @@
       <c r="D6" s="5"/>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" spans="1:5">
+    <row r="7" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
         <v>13</v>
       </c>
@@ -704,7 +733,7 @@
       <c r="D7" s="5"/>
       <c r="E7" s="5"/>
     </row>
-    <row r="8" spans="1:5">
+    <row r="8" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A8" s="4" t="s">
         <v>16</v>
       </c>
@@ -717,7 +746,7 @@
       <c r="D8" s="5"/>
       <c r="E8" s="5"/>
     </row>
-    <row r="9" spans="1:5">
+    <row r="9" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="4" t="s">
         <v>19</v>
       </c>
@@ -730,7 +759,7 @@
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
     </row>
-    <row r="10" spans="1:5">
+    <row r="10" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="4" t="s">
         <v>22</v>
       </c>
@@ -743,7 +772,7 @@
       <c r="D10" s="5"/>
       <c r="E10" s="5"/>
     </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="4" t="s">
         <v>25</v>
       </c>
@@ -756,7 +785,7 @@
       <c r="D11" s="5"/>
       <c r="E11" s="5"/>
     </row>
-    <row r="12" spans="1:5">
+    <row r="12" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="4" t="s">
         <v>28</v>
       </c>
@@ -769,7 +798,7 @@
       <c r="D12" s="5"/>
       <c r="E12" s="5"/>
     </row>
-    <row r="13" spans="1:5">
+    <row r="13" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="4" t="s">
         <v>31</v>
       </c>
@@ -782,7 +811,7 @@
       <c r="D13" s="5"/>
       <c r="E13" s="5"/>
     </row>
-    <row r="14" spans="1:5">
+    <row r="14" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A14" s="4" t="s">
         <v>34</v>
       </c>
@@ -795,7 +824,7 @@
       <c r="D14" s="5"/>
       <c r="E14" s="5"/>
     </row>
-    <row r="15" spans="1:5">
+    <row r="15" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="4" t="s">
         <v>37</v>
       </c>
@@ -808,7 +837,7 @@
       <c r="D15" s="5"/>
       <c r="E15" s="5"/>
     </row>
-    <row r="16" spans="1:5">
+    <row r="16" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A16" s="4" t="s">
         <v>40</v>
       </c>
@@ -821,7 +850,7 @@
       <c r="D16" s="5"/>
       <c r="E16" s="5"/>
     </row>
-    <row r="17" spans="1:5">
+    <row r="17" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="4" t="s">
         <v>43</v>
       </c>
@@ -834,7 +863,7 @@
       <c r="D17" s="5"/>
       <c r="E17" s="5"/>
     </row>
-    <row r="18" spans="1:5">
+    <row r="18" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="4" t="s">
         <v>46</v>
       </c>
@@ -847,7 +876,7 @@
       <c r="D18" s="5"/>
       <c r="E18" s="5"/>
     </row>
-    <row r="19" spans="1:5">
+    <row r="19" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="4" t="s">
         <v>49</v>
       </c>
@@ -860,7 +889,7 @@
       <c r="D19" s="5"/>
       <c r="E19" s="5"/>
     </row>
-    <row r="20" spans="1:5">
+    <row r="20" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="4" t="s">
         <v>52</v>
       </c>
@@ -873,7 +902,7 @@
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
     </row>
-    <row r="21" spans="1:5">
+    <row r="21" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="4" t="s">
         <v>55</v>
       </c>
@@ -886,7 +915,7 @@
       <c r="D21" s="5"/>
       <c r="E21" s="5"/>
     </row>
-    <row r="22" spans="1:5">
+    <row r="22" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A22" s="4" t="s">
         <v>58</v>
       </c>
@@ -899,7 +928,7 @@
       <c r="D22" s="5"/>
       <c r="E22" s="5"/>
     </row>
-    <row r="23" spans="1:5">
+    <row r="23" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A23" s="4" t="s">
         <v>61</v>
       </c>
@@ -912,7 +941,7 @@
       <c r="D23" s="5"/>
       <c r="E23" s="5"/>
     </row>
-    <row r="24" spans="1:5">
+    <row r="24" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="4" t="s">
         <v>64</v>
       </c>
@@ -925,7 +954,7 @@
       <c r="D24" s="5"/>
       <c r="E24" s="5"/>
     </row>
-    <row r="25" spans="1:5">
+    <row r="25" spans="1:5" ht="16" x14ac:dyDescent="0.2">
       <c r="A25" s="4" t="s">
         <v>67</v>
       </c>
@@ -938,7 +967,7 @@
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
     </row>
-    <row r="26" spans="1:5">
+    <row r="26" spans="1:5" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="4" t="s">
         <v>70</v>
       </c>
@@ -953,7 +982,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D26">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D5:D26" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Pass,Fail,Partial"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>